<commit_message>
feat(data): accumulate fact table across months instead of rebuilding
The ENAP source is a rolling 12-month dump, so rebuilding dashboard_base.csv
from scratch each run silently dropped the months that fell out of the
window (cumulative totals shifted week to week). Add an idempotent monthly
merge (merge_fato) that preserves months outside the current download and
replaces only the months present in it, plus a --rebuild flag to force a
full rebuild. Mirrors the merge pattern already used in atualizar_historico.py.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/relatorio_capacitacao_ia.xlsx
+++ b/docs/relatorio_capacitacao_ia.xlsx
@@ -519,7 +519,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Data: 27/05/2026  ·  Período coberto: 2024-08 a 2026-04  ·  Fonte: dadosaberto.evg.gov.br</t>
+          <t>Data: 02/06/2026  ·  Período coberto: 2025-06 a 2026-05  ·  Fonte: dadosaberto.evg.gov.br</t>
         </is>
       </c>
     </row>
@@ -557,16 +557,16 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>161712</v>
+        <v>117117</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>53087</v>
+        <v>34634</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>272383</v>
+        <v>191371</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>86794</v>
+        <v>54394</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>68065</v>
+        <v>47328</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>28263</v>
+        <v>19816</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>116148</v>
+        <v>77648</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>49179</v>
+        <v>32863</v>
       </c>
     </row>
     <row r="8">
@@ -606,16 +606,16 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>76107</v>
+        <v>58824</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>18001</v>
+        <v>10843</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>129788</v>
+        <v>97887</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>27584</v>
+        <v>15980</v>
       </c>
     </row>
     <row r="9">
@@ -625,16 +625,16 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>17989</v>
+        <v>11202</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>6950</v>
+        <v>4029</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>26447</v>
+        <v>15836</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>10031</v>
+        <v>5551</v>
       </c>
     </row>
     <row r="10">
@@ -655,16 +655,16 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>83434</v>
+        <v>60799</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>28593</v>
+        <v>19025</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>149611</v>
+        <v>105041</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>47989</v>
+        <v>30577</v>
       </c>
     </row>
     <row r="12">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>2151</v>
+        <v>1354</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>938</v>
+        <v>527</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>3630</v>
+        <v>2183</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>1519</v>
+        <v>836</v>
       </c>
     </row>
     <row r="13">
@@ -693,16 +693,16 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>16016</v>
+        <v>10279</v>
       </c>
       <c r="C13" s="10" t="n">
-        <v>8212</v>
+        <v>4783</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>25662</v>
+        <v>15694</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>12904</v>
+        <v>7520</v>
       </c>
     </row>
     <row r="14">
@@ -712,16 +712,16 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>61881</v>
+        <v>45952</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>15623</v>
+        <v>10447</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>93480</v>
+        <v>68453</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>24382</v>
+        <v>15461</v>
       </c>
     </row>
     <row r="15">
@@ -731,16 +731,16 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>86181</v>
+        <v>52525</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>29444</v>
+        <v>16429</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>112776</v>
+        <v>67623</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>38579</v>
+        <v>21119</v>
       </c>
     </row>
     <row r="16">
@@ -750,22 +750,22 @@
         </is>
       </c>
       <c r="B16" s="14" t="n">
-        <v>247081</v>
+        <v>169216</v>
       </c>
       <c r="C16" s="14" t="n">
-        <v>82349</v>
+        <v>50975</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>385159</v>
+        <v>258994</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>125373</v>
+        <v>75513</v>
       </c>
     </row>
     <row r="18" ht="70" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Pessoas = contagem única de pessoas (codigo_pessoa); NÃO somam entre grupos. Matrículas = nº de conclusões (somam). Federal+Estadual+Municipal reconciliam o total público em matrículas; os poderes não (~32% dos registros públicos sem poder informado). "Setor Privado / não-servidor" agrega iniciativa privada, sociedade civil e público geral. Filtros: sit_matricula=Concluida; 35 cursos-alvo; dt_matricula em [2024-08, 2026-04].</t>
+          <t>Pessoas = contagem única de pessoas (codigo_pessoa); NÃO somam entre grupos. Matrículas = nº de conclusões (somam). Federal+Estadual+Municipal reconciliam o total público em matrículas; os poderes não (~32% dos registros públicos sem poder informado). "Setor Privado / não-servidor" agrega iniciativa privada, sociedade civil e público geral. Filtros: sit_matricula=Concluida; 35 cursos-alvo; dt_matricula em [2024-08, 2026-05].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(pbip): aprimora dashboard com filtros, titulos, rotulos e cultura pt-BR
- Filtros, titulos de pagina e rotulos nos visuais das 3 paginas
- Top-10 de cursos e tabela de cursos
- Cultura pt-BR no modelo semantico
- Base do dashboard (dashboard_base.csv) e ajustes no gerador
- .gitignore: whitelist do dashboard_base.csv e backups datados

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/relatorio_capacitacao_ia.xlsx
+++ b/docs/relatorio_capacitacao_ia.xlsx
@@ -519,7 +519,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Data: 02/06/2026  ·  Período coberto: 2025-06 a 2026-05  ·  Fonte: dadosaberto.evg.gov.br</t>
+          <t>Data: 09/06/2026  ·  Período coberto: 2024-08 a 2026-05  ·  Fonte: dadosaberto.evg.gov.br</t>
         </is>
       </c>
     </row>
@@ -557,16 +557,16 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>117117</v>
+        <v>167284</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>34634</v>
+        <v>55577</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>191371</v>
+        <v>282957</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>54394</v>
+        <v>91004</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>47328</v>
+        <v>71101</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>19816</v>
+        <v>29734</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>77648</v>
+        <v>122400</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>32863</v>
+        <v>51837</v>
       </c>
     </row>
     <row r="8">
@@ -606,16 +606,16 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>58824</v>
+        <v>77891</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>10843</v>
+        <v>18707</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>97887</v>
+        <v>132866</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>15980</v>
+        <v>28661</v>
       </c>
     </row>
     <row r="9">
@@ -625,16 +625,16 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>11202</v>
+        <v>18777</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>4029</v>
+        <v>7274</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>15836</v>
+        <v>27691</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>5551</v>
+        <v>10506</v>
       </c>
     </row>
     <row r="10">
@@ -655,16 +655,16 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>60799</v>
+        <v>86507</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>19025</v>
+        <v>30053</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>105041</v>
+        <v>155744</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>30577</v>
+        <v>50507</v>
       </c>
     </row>
     <row r="12">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>1354</v>
+        <v>2240</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>527</v>
+        <v>979</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>2183</v>
+        <v>3770</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>836</v>
+        <v>1580</v>
       </c>
     </row>
     <row r="13">
@@ -693,16 +693,16 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>10279</v>
+        <v>16701</v>
       </c>
       <c r="C13" s="10" t="n">
-        <v>4783</v>
+        <v>8469</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>15694</v>
+        <v>26867</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>7520</v>
+        <v>13338</v>
       </c>
     </row>
     <row r="14">
@@ -712,16 +712,16 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>45952</v>
+        <v>63678</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>10447</v>
+        <v>16376</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>68453</v>
+        <v>96576</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>15461</v>
+        <v>25579</v>
       </c>
     </row>
     <row r="15">
@@ -731,16 +731,16 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>52525</v>
+        <v>90878</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>16429</v>
+        <v>30690</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>67623</v>
+        <v>119287</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>21119</v>
+        <v>40288</v>
       </c>
     </row>
     <row r="16">
@@ -750,16 +750,16 @@
         </is>
       </c>
       <c r="B16" s="14" t="n">
-        <v>169216</v>
+        <v>257295</v>
       </c>
       <c r="C16" s="14" t="n">
-        <v>50975</v>
+        <v>86076</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>258994</v>
+        <v>402244</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>75513</v>
+        <v>131292</v>
       </c>
     </row>
     <row r="18" ht="70" customHeight="1">

</xml_diff>

<commit_message>
feat(pbip): add June 2026 data and Programa dimension
Data refresh:
- Regenerate dashboard from ENAP "last 12 months" dump (2026-07-01),
  adding closed June 2026. Fact table now spans 2024-08..2026-06
  (421,340 rows); June has 15,457 enrollments across the 35 target courses.

Programa dimension (course->programa bridge, m:n):
- New pages 07-por-programa and 08-distribuicao-programa
- New bridge_programa / dist_programa tables + generator gerar_programa.py
- Curated source scripts/cursos_programa.csv (now whitelisted in .gitignore
  so the feature is reproducible)

PBIP uses relative CsvPath (repo default); regenerate locally with
--csv-path-mode absolute to open in Power BI Desktop.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/relatorio_capacitacao_ia.xlsx
+++ b/docs/relatorio_capacitacao_ia.xlsx
@@ -519,7 +519,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Data: 09/06/2026  ·  Período coberto: 2024-08 a 2026-05  ·  Fonte: dadosaberto.evg.gov.br</t>
+          <t>Data: 08/07/2026  ·  Período coberto: 2024-08 a 2026-06  ·  Fonte: dadosaberto.evg.gov.br</t>
         </is>
       </c>
     </row>
@@ -557,16 +557,16 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>167284</v>
+        <v>173553</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>55577</v>
+        <v>58016</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>282957</v>
+        <v>294271</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>91004</v>
+        <v>95145</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>71101</v>
+        <v>74764</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>29734</v>
+        <v>31093</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>122400</v>
+        <v>129295</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>51837</v>
+        <v>54348</v>
       </c>
     </row>
     <row r="8">
@@ -606,16 +606,16 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>77891</v>
+        <v>79713</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>18707</v>
+        <v>19427</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>132866</v>
+        <v>135940</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>28661</v>
+        <v>29748</v>
       </c>
     </row>
     <row r="9">
@@ -625,16 +625,16 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>18777</v>
+        <v>19609</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>7274</v>
+        <v>7643</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>27691</v>
+        <v>29036</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>10506</v>
+        <v>11049</v>
       </c>
     </row>
     <row r="10">
@@ -655,16 +655,16 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>86507</v>
+        <v>90243</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>30053</v>
+        <v>31522</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>155744</v>
+        <v>162638</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>50507</v>
+        <v>53054</v>
       </c>
     </row>
     <row r="12">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>2240</v>
+        <v>2325</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>979</v>
+        <v>1019</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>3770</v>
+        <v>3912</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>1580</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="13">
@@ -693,16 +693,16 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>16701</v>
+        <v>17285</v>
       </c>
       <c r="C13" s="10" t="n">
-        <v>8469</v>
+        <v>8675</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>26867</v>
+        <v>27928</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>13338</v>
+        <v>13686</v>
       </c>
     </row>
     <row r="14">
@@ -712,16 +712,16 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>63678</v>
+        <v>65621</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>16376</v>
+        <v>17115</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>96576</v>
+        <v>99793</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>25579</v>
+        <v>26756</v>
       </c>
     </row>
     <row r="15">
@@ -731,16 +731,16 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>90878</v>
+        <v>96768</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>30690</v>
+        <v>31797</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>119287</v>
+        <v>127069</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>40288</v>
+        <v>41796</v>
       </c>
     </row>
     <row r="16">
@@ -750,22 +750,22 @@
         </is>
       </c>
       <c r="B16" s="14" t="n">
-        <v>257295</v>
+        <v>269350</v>
       </c>
       <c r="C16" s="14" t="n">
-        <v>86076</v>
+        <v>89611</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>402244</v>
+        <v>421340</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>131292</v>
+        <v>136941</v>
       </c>
     </row>
     <row r="18" ht="70" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Pessoas = contagem única de pessoas (codigo_pessoa); NÃO somam entre grupos. Matrículas = nº de conclusões (somam). Federal+Estadual+Municipal reconciliam o total público em matrículas; os poderes não (~32% dos registros públicos sem poder informado). "Setor Privado / não-servidor" agrega iniciativa privada, sociedade civil e público geral. Filtros: sit_matricula=Concluida; 35 cursos-alvo; dt_matricula em [2024-08, 2026-05].</t>
+          <t>Pessoas = contagem única de pessoas (codigo_pessoa); NÃO somam entre grupos. Matrículas = nº de conclusões (somam). Federal+Estadual+Municipal reconciliam o total público em matrículas; os poderes não (~32% dos registros públicos sem poder informado). "Setor Privado / não-servidor" agrega iniciativa privada, sociedade civil e público geral. Filtros: sit_matricula=Concluida; 35 cursos-alvo; dt_matricula em [2024-08, 2026-06].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(historico): atualizacao automatica 2026-09-01
</commit_message>
<xml_diff>
--- a/docs/relatorio_capacitacao_ia.xlsx
+++ b/docs/relatorio_capacitacao_ia.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Indicadores" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -519,7 +519,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Data: 15/07/2026  ·  Período coberto: 2024-08 a 2026-06  ·  Fonte: dadosaberto.evg.gov.br</t>
+          <t>Data: 01/09/2026  ·  Período coberto: 2024-08 a 2026-07  ·  Fonte: dadosaberto.evg.gov.br</t>
         </is>
       </c>
     </row>
@@ -557,16 +557,16 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>95145</v>
+        <v>101137</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>132596</v>
+        <v>138774</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>58016</v>
+        <v>61510</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>90578</v>
+        <v>95175</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>54348</v>
+        <v>58088</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>35481</v>
+        <v>38470</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>31093</v>
+        <v>33073</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>27418</v>
+        <v>29484</v>
       </c>
     </row>
     <row r="8">
@@ -606,16 +606,16 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>29748</v>
+        <v>31213</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>87383</v>
+        <v>89995</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>19427</v>
+        <v>20400</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>55359</v>
+        <v>57468</v>
       </c>
     </row>
     <row r="9">
@@ -625,16 +625,16 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>11049</v>
+        <v>11836</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>9732</v>
+        <v>10309</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>7643</v>
+        <v>8195</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>7968</v>
+        <v>8403</v>
       </c>
     </row>
     <row r="10">
@@ -655,16 +655,16 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>53054</v>
+        <v>56877</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>77958</v>
+        <v>82007</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>31522</v>
+        <v>33757</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>53041</v>
+        <v>56079</v>
       </c>
     </row>
     <row r="12">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>1649</v>
+        <v>1746</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>1451</v>
+        <v>1532</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>1019</v>
+        <v>1079</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>1065</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="13">
@@ -693,16 +693,16 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>13686</v>
+        <v>14209</v>
       </c>
       <c r="C13" s="10" t="n">
-        <v>7919</v>
+        <v>8404</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>8675</v>
+        <v>9011</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>6567</v>
+        <v>6954</v>
       </c>
     </row>
     <row r="14">
@@ -712,16 +712,16 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>26756</v>
+        <v>28305</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>45268</v>
+        <v>46831</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>17115</v>
+        <v>18012</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>31038</v>
+        <v>32194</v>
       </c>
     </row>
     <row r="15">
@@ -731,16 +731,16 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>41796</v>
+        <v>43924</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>45246</v>
+        <v>48168</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>31797</v>
+        <v>33200</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>38454</v>
+        <v>40751</v>
       </c>
     </row>
     <row r="16">
@@ -750,22 +750,22 @@
         </is>
       </c>
       <c r="B16" s="14" t="n">
-        <v>136941</v>
+        <v>145061</v>
       </c>
       <c r="C16" s="14" t="n">
-        <v>177842</v>
+        <v>186942</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>89611</v>
+        <v>94492</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>128704</v>
+        <v>135573</v>
       </c>
     </row>
     <row r="18" ht="70" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Indicadores cobrem apenas IA e Dados (Gestão e Outros ficam de fora). Pessoas = contagem única de pessoas (codigo_pessoa); NÃO somam entre grupos. Matrículas = nº de conclusões (somam). Federal+Estadual+Municipal reconciliam o total público em matrículas; os poderes não (~32% dos registros públicos sem poder informado). "Setor Privado / não-servidor" agrega iniciativa privada, sociedade civil e público geral. Filtros: sit_matricula=Concluida; 35 cursos-alvo; dt_matricula em [2024-08, 2026-06].</t>
+          <t>Indicadores cobrem apenas IA e Dados (Gestão e Outros ficam de fora). Pessoas = contagem única de pessoas (codigo_pessoa); NÃO somam entre grupos. Matrículas = nº de conclusões (somam). Federal+Estadual+Municipal reconciliam o total público em matrículas; os poderes não (~32% dos registros públicos sem poder informado). "Setor Privado / não-servidor" agrega iniciativa privada, sociedade civil e público geral. Filtros: sit_matricula=Concluida; 35 cursos-alvo; dt_matricula em [2024-08, 2026-08].</t>
         </is>
       </c>
     </row>

</xml_diff>